<commit_message>
Updated IND_grids_kan model - 2026-06-12 15:43
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B56E0341-F974-4E82-BEE7-72529803C937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{828D8638-AECA-426A-8426-9CD81DC6EF55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6694,7 +6694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58C643C8-72C5-4CF5-A8BE-53E7B0D3D532}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DF51B57-493A-47E4-A896-379F35950BBB}">
   <dimension ref="B9:H527"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -37267,7 +37267,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{583AF7D4-4150-4C51-9E14-DC6241BE583A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D389D56B-B927-475C-BFD8-4A9437C6D9A0}">
   <dimension ref="B9:L527"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>